<commit_message>
testing stuff + phase 15
</commit_message>
<xml_diff>
--- a/ev_chargers_islington_city_centre_west.xlsx
+++ b/ev_chargers_islington_city_centre_west.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sujal\hackathons\wattif-clean\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76C9A296-A7A4-4265-ACD8-61293C1F1CB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D39B50F-F62D-4C91-8710-A020BFC52D64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21697" yWindow="-98" windowWidth="21795" windowHeight="13695" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="26">
   <si>
     <t>latitude</t>
   </si>
@@ -36,46 +36,73 @@
     <t>charger_type</t>
   </si>
   <si>
-    <t>ports</t>
-  </si>
-  <si>
-    <t>average_daily_sessions</t>
-  </si>
-  <si>
-    <t>complaints</t>
-  </si>
-  <si>
-    <t>station_name</t>
-  </si>
-  <si>
-    <t>Kipling Station Hub</t>
-  </si>
-  <si>
-    <t>DC Fast</t>
-  </si>
-  <si>
-    <t>Commuters say chargers are usually full during evening rush</t>
-  </si>
-  <si>
-    <t>Six Points Plaza</t>
-  </si>
-  <si>
     <t>Level 2</t>
   </si>
   <si>
-    <t>Residents want more chargers near grocery stores and shops</t>
-  </si>
-  <si>
-    <t>Islington Village</t>
-  </si>
-  <si>
-    <t>Drivers say charging access is limited west of Islington</t>
-  </si>
-  <si>
-    <t>Cloverdale Mall Area</t>
-  </si>
-  <si>
-    <t>EV owners want chargers closer to mall entrances</t>
+    <t>name</t>
+  </si>
+  <si>
+    <t>address</t>
+  </si>
+  <si>
+    <t>power_kw</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>operator</t>
+  </si>
+  <si>
+    <t>Islington Charger A</t>
+  </si>
+  <si>
+    <t>100 City Centre Dr</t>
+  </si>
+  <si>
+    <t>Level 3</t>
+  </si>
+  <si>
+    <t>active</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>Islington Charger B</t>
+  </si>
+  <si>
+    <t>5242 Dundas St W</t>
+  </si>
+  <si>
+    <t>Private</t>
+  </si>
+  <si>
+    <t>Islington Charger C</t>
+  </si>
+  <si>
+    <t>399 The West Mall</t>
+  </si>
+  <si>
+    <t>unavailable</t>
+  </si>
+  <si>
+    <t>Utility</t>
+  </si>
+  <si>
+    <t>Islington Charger D</t>
+  </si>
+  <si>
+    <t>10 East Mall Crescent</t>
+  </si>
+  <si>
+    <t>Islington Charger E</t>
+  </si>
+  <si>
+    <t>250 The East Mall</t>
+  </si>
+  <si>
+    <t>maintenance</t>
   </si>
 </sst>
 </file>
@@ -393,129 +420,170 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.06640625" customWidth="1"/>
-    <col min="2" max="2" width="7.73046875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.06640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.33203125" customWidth="1"/>
-    <col min="7" max="7" width="48.9296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="36.28515625" customWidth="1"/>
+    <col min="2" max="2" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" customWidth="1"/>
+    <col min="7" max="7" width="49" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2">
+        <v>43.645200000000003</v>
+      </c>
+      <c r="D2">
+        <v>-79.528099999999995</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2">
+        <v>150</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3">
+        <v>43.637799999999999</v>
+      </c>
+      <c r="D3">
+        <v>-79.536900000000003</v>
+      </c>
+      <c r="E3" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2">
-        <v>43.637300000000003</v>
-      </c>
-      <c r="C2">
-        <v>-79.535700000000006</v>
-      </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2">
-        <v>6</v>
-      </c>
-      <c r="F2">
-        <v>58</v>
-      </c>
-      <c r="G2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3">
-        <v>43.642200000000003</v>
-      </c>
-      <c r="C3">
-        <v>-79.531800000000004</v>
-      </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3">
-        <v>8</v>
-      </c>
       <c r="F3">
-        <v>44</v>
+        <v>19.2</v>
       </c>
       <c r="G3" t="s">
         <v>12</v>
       </c>
+      <c r="H3" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4">
+        <v>43.6494</v>
+      </c>
+      <c r="D4">
+        <v>-79.559100000000001</v>
+      </c>
+      <c r="E4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4">
+        <v>100</v>
+      </c>
+      <c r="G4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5">
+        <v>43.630800000000001</v>
+      </c>
+      <c r="D5">
+        <v>-79.553200000000004</v>
+      </c>
+      <c r="E5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F5">
+        <v>22</v>
+      </c>
+      <c r="G5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" t="s">
         <v>13</v>
       </c>
-      <c r="B4">
-        <v>43.645000000000003</v>
-      </c>
-      <c r="C4">
-        <v>-79.524000000000001</v>
-      </c>
-      <c r="D4" t="s">
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6">
+        <v>43.642099999999999</v>
+      </c>
+      <c r="D6">
+        <v>-79.558700000000002</v>
+      </c>
+      <c r="E6" t="s">
         <v>11</v>
       </c>
-      <c r="E4">
-        <v>4</v>
-      </c>
-      <c r="F4">
+      <c r="F6">
+        <v>120</v>
+      </c>
+      <c r="G6" t="s">
         <v>25</v>
       </c>
-      <c r="G4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5">
-        <v>43.6325</v>
-      </c>
-      <c r="C5">
-        <v>-79.5565</v>
-      </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5">
-        <v>10</v>
-      </c>
-      <c r="F5">
-        <v>62</v>
-      </c>
-      <c r="G5" t="s">
-        <v>16</v>
+      <c r="H6" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>